<commit_message>
fix(desocup): corrige agregación de tasas mensuales y etiquetas trimestrales.
- build_data.py: is_quarter ahora usa el FREQ de la serie (string "4") en lugar
de ind.frecuencia, evitando que las tasas mensuales de ENOE se colapsen a trimestres.
- build_data.py: agrega q_period a observaciones con población ocupada.
- assets/js/metrics.js: usa q_period para el dato trimestral de población ocupada.
- assets/js/charts.js: eje x de población ocupada usa q_period.
- Regenera datos online: 102 observaciones mensuales, población ocupada trimestral
hasta 2T-26 (60.04 millones), 4 tasas hasta Jun 26.

Generated with Devin

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/DESOCUP/DESOCUP_datos.xlsx
+++ b/downloads/indicadores/DESOCUP/DESOCUP_datos.xlsx
@@ -571,11 +571,17 @@
         <v>43101</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>3.3645</v>
-      </c>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
+        <v>3.364517</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>59.046013</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>56.916034</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>7.000563</v>
+      </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -607,11 +613,17 @@
         <v>43132</v>
       </c>
       <c r="C6" s="8" t="n">
-        <v>3.1736</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
+        <v>3.173574</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>59.209673</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>56.354829</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>6.266172</v>
+      </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -643,11 +655,17 @@
         <v>43160</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>2.9372</v>
-      </c>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
+        <v>2.937211</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>59.113431</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>56.480453</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>6.84393</v>
+      </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -679,11 +697,17 @@
         <v>43191</v>
       </c>
       <c r="C8" s="8" t="n">
-        <v>3.3865</v>
-      </c>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
+        <v>3.386516</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>59.481548</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>56.440433</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>7.11</v>
+      </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -715,11 +739,17 @@
         <v>43221</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>3.2237</v>
-      </c>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
+        <v>3.223703</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>60.152678</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>56.617137</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>7.102237</v>
+      </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -751,11 +781,17 @@
         <v>43252</v>
       </c>
       <c r="C10" s="8" t="n">
-        <v>3.3735</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
+        <v>3.373504</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>59.844343</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>56.320885</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>6.693838</v>
+      </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -787,11 +823,17 @@
         <v>43282</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>3.4721</v>
-      </c>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
+        <v>3.472051</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>59.791741</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>56.753537</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>7.106279</v>
+      </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -823,11 +865,17 @@
         <v>43313</v>
       </c>
       <c r="C12" s="8" t="n">
-        <v>3.4573</v>
-      </c>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
+        <v>3.45726</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>60.054514</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>56.695026</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>7.373657</v>
+      </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -859,11 +907,17 @@
         <v>43344</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>3.5812</v>
-      </c>
-      <c r="D13" s="6" t="n"/>
-      <c r="E13" s="6" t="n"/>
-      <c r="F13" s="6" t="n"/>
+        <v>3.581227</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>59.598593</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>56.155985</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>6.637874</v>
+      </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -895,11 +949,17 @@
         <v>43374</v>
       </c>
       <c r="C14" s="8" t="n">
-        <v>3.2659</v>
-      </c>
-      <c r="D14" s="8" t="n"/>
-      <c r="E14" s="8" t="n"/>
-      <c r="F14" s="8" t="n"/>
+        <v>3.265938</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>59.420827</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>55.808527</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>6.900635</v>
+      </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -931,11 +991,17 @@
         <v>43405</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>3.2485</v>
-      </c>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
+        <v>3.248481</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>60.027049</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>57.064916</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>6.834767</v>
+      </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -967,11 +1033,17 @@
         <v>43435</v>
       </c>
       <c r="C16" s="8" t="n">
-        <v>3.3584</v>
-      </c>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
+        <v>3.358366</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>59.522655</v>
+      </c>
+      <c r="E16" s="8" t="n">
+        <v>56.584476</v>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>6.494008</v>
+      </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1003,11 +1075,17 @@
         <v>43466</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>3.5633</v>
-      </c>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
+        <v>3.563302</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>59.306168</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>56.464509</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>6.80502</v>
+      </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1039,11 +1117,17 @@
         <v>43497</v>
       </c>
       <c r="C18" s="8" t="n">
-        <v>3.2936</v>
-      </c>
-      <c r="D18" s="8" t="n"/>
-      <c r="E18" s="8" t="n"/>
-      <c r="F18" s="8" t="n"/>
+        <v>3.293564</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>59.298864</v>
+      </c>
+      <c r="E18" s="8" t="n">
+        <v>57.499623</v>
+      </c>
+      <c r="F18" s="8" t="n">
+        <v>6.315581</v>
+      </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1075,11 +1159,17 @@
         <v>43525</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>3.2239</v>
-      </c>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
+        <v>3.223913</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>60.053019</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>56.533358</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>6.804934</v>
+      </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1111,11 +1201,17 @@
         <v>43556</v>
       </c>
       <c r="C20" s="8" t="n">
-        <v>3.4985</v>
-      </c>
-      <c r="D20" s="8" t="n"/>
-      <c r="E20" s="8" t="n"/>
-      <c r="F20" s="8" t="n"/>
+        <v>3.498489</v>
+      </c>
+      <c r="D20" s="8" t="n">
+        <v>59.758411</v>
+      </c>
+      <c r="E20" s="8" t="n">
+        <v>56.24954</v>
+      </c>
+      <c r="F20" s="8" t="n">
+        <v>7.740641</v>
+      </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1147,11 +1243,17 @@
         <v>43586</v>
       </c>
       <c r="C21" s="6" t="n">
-        <v>3.502</v>
-      </c>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
+        <v>3.501957</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>60.253945</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>56.034385</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>7.685463</v>
+      </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1183,11 +1285,17 @@
         <v>43617</v>
       </c>
       <c r="C22" s="8" t="n">
-        <v>3.5652</v>
-      </c>
-      <c r="D22" s="8" t="n"/>
-      <c r="E22" s="8" t="n"/>
-      <c r="F22" s="8" t="n"/>
+        <v>3.56515</v>
+      </c>
+      <c r="D22" s="8" t="n">
+        <v>60.575741</v>
+      </c>
+      <c r="E22" s="8" t="n">
+        <v>56.232594</v>
+      </c>
+      <c r="F22" s="8" t="n">
+        <v>7.475064</v>
+      </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1219,11 +1327,17 @@
         <v>43647</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>3.7368</v>
-      </c>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
+        <v>3.736801</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>60.54807</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>56.103232</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>7.83611</v>
+      </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1255,11 +1369,17 @@
         <v>43678</v>
       </c>
       <c r="C24" s="8" t="n">
-        <v>3.7067</v>
-      </c>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="8" t="n"/>
+        <v>3.706726</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <v>60.477838</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>56.286051</v>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>7.431028</v>
+      </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1291,11 +1411,17 @@
         <v>43709</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>3.7809</v>
-      </c>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
+        <v>3.780859</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>60.169709</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>56.481424</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>7.801007</v>
+      </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1327,11 +1453,17 @@
         <v>43739</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>3.6914</v>
-      </c>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="n"/>
+        <v>3.691382</v>
+      </c>
+      <c r="D26" s="8" t="n">
+        <v>60.292051</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <v>56.043479</v>
+      </c>
+      <c r="F26" s="8" t="n">
+        <v>7.706281</v>
+      </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1363,11 +1495,17 @@
         <v>43770</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>3.4182</v>
-      </c>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
+        <v>3.418223</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>60.618629</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>55.949132</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>8.162853</v>
+      </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1399,11 +1537,17 @@
         <v>43800</v>
       </c>
       <c r="C28" s="8" t="n">
-        <v>2.9052</v>
-      </c>
-      <c r="D28" s="8" t="n"/>
-      <c r="E28" s="8" t="n"/>
-      <c r="F28" s="8" t="n"/>
+        <v>2.905177</v>
+      </c>
+      <c r="D28" s="8" t="n">
+        <v>60.202267</v>
+      </c>
+      <c r="E28" s="8" t="n">
+        <v>55.985652</v>
+      </c>
+      <c r="F28" s="8" t="n">
+        <v>6.937417</v>
+      </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1435,11 +1579,17 @@
         <v>43831</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>3.7797</v>
-      </c>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
+        <v>3.779704</v>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>59.821448</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>56.090148</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>7.385867</v>
+      </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1471,11 +1621,17 @@
         <v>43862</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>3.5302</v>
-      </c>
-      <c r="D30" s="8" t="n"/>
-      <c r="E30" s="8" t="n"/>
-      <c r="F30" s="8" t="n"/>
+        <v>3.530188</v>
+      </c>
+      <c r="D30" s="8" t="n">
+        <v>60.178852</v>
+      </c>
+      <c r="E30" s="8" t="n">
+        <v>56.106063</v>
+      </c>
+      <c r="F30" s="8" t="n">
+        <v>8.632664999999999</v>
+      </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1507,11 +1663,17 @@
         <v>43891</v>
       </c>
       <c r="C31" s="6" t="n">
-        <v>2.909</v>
-      </c>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
+        <v>2.908969</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>59.807992</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>55.537911</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>9.059552</v>
+      </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1543,11 +1705,17 @@
         <v>43922</v>
       </c>
       <c r="C32" s="8" t="n">
-        <v>4.6864</v>
-      </c>
-      <c r="D32" s="8" t="n"/>
-      <c r="E32" s="8" t="n"/>
-      <c r="F32" s="8" t="n"/>
+        <v>4.686441</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>47.17972</v>
+      </c>
+      <c r="E32" s="8" t="n">
+        <v>47.887397</v>
+      </c>
+      <c r="F32" s="8" t="n">
+        <v>25.40378</v>
+      </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1579,11 +1747,17 @@
         <v>43952</v>
       </c>
       <c r="C33" s="6" t="n">
-        <v>4.1928</v>
-      </c>
-      <c r="D33" s="6" t="n"/>
-      <c r="E33" s="6" t="n"/>
-      <c r="F33" s="6" t="n"/>
+        <v>4.192756</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>47.447129</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>51.836731</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>29.94159</v>
+      </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1615,11 +1789,17 @@
         <v>43983</v>
       </c>
       <c r="C34" s="8" t="n">
-        <v>5.4922</v>
-      </c>
-      <c r="D34" s="8" t="n"/>
-      <c r="E34" s="8" t="n"/>
-      <c r="F34" s="8" t="n"/>
+        <v>5.492159</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <v>53.111205</v>
+      </c>
+      <c r="E34" s="8" t="n">
+        <v>53.027107</v>
+      </c>
+      <c r="F34" s="8" t="n">
+        <v>20.051608</v>
+      </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1651,11 +1831,17 @@
         <v>44013</v>
       </c>
       <c r="C35" s="6" t="n">
-        <v>5.3509</v>
-      </c>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
+        <v>5.350869</v>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>54.992563</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>54.979852</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>18.339857</v>
+      </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1687,11 +1873,17 @@
         <v>44044</v>
       </c>
       <c r="C36" s="8" t="n">
-        <v>5.2575</v>
-      </c>
-      <c r="D36" s="8" t="n"/>
-      <c r="E36" s="8" t="n"/>
-      <c r="F36" s="8" t="n"/>
+        <v>5.257507</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <v>55.123265</v>
+      </c>
+      <c r="E36" s="8" t="n">
+        <v>55.00344</v>
+      </c>
+      <c r="F36" s="8" t="n">
+        <v>16.861652</v>
+      </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1723,11 +1915,17 @@
         <v>44075</v>
       </c>
       <c r="C37" s="6" t="n">
-        <v>5.1285</v>
-      </c>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
+        <v>5.12847</v>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>55.688833</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>54.887539</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>15.574149</v>
+      </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1759,11 +1957,17 @@
         <v>44105</v>
       </c>
       <c r="C38" s="8" t="n">
-        <v>4.7085</v>
-      </c>
-      <c r="D38" s="8" t="n"/>
-      <c r="E38" s="8" t="n"/>
-      <c r="F38" s="8" t="n"/>
+        <v>4.708477</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <v>57.477385</v>
+      </c>
+      <c r="E38" s="8" t="n">
+        <v>55.86088</v>
+      </c>
+      <c r="F38" s="8" t="n">
+        <v>14.889134</v>
+      </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1795,11 +1999,17 @@
         <v>44136</v>
       </c>
       <c r="C39" s="6" t="n">
-        <v>4.3537</v>
-      </c>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
+        <v>4.353693</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>56.928332</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>56.18434</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>15.803526</v>
+      </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1831,11 +2041,17 @@
         <v>44166</v>
       </c>
       <c r="C40" s="8" t="n">
-        <v>3.7904</v>
-      </c>
-      <c r="D40" s="8" t="n"/>
-      <c r="E40" s="8" t="n"/>
-      <c r="F40" s="8" t="n"/>
+        <v>3.790374</v>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>56.515036</v>
+      </c>
+      <c r="E40" s="8" t="n">
+        <v>55.667354</v>
+      </c>
+      <c r="F40" s="8" t="n">
+        <v>14.117299</v>
+      </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1867,11 +2083,17 @@
         <v>44197</v>
       </c>
       <c r="C41" s="6" t="n">
-        <v>4.7027</v>
-      </c>
-      <c r="D41" s="6" t="n"/>
-      <c r="E41" s="6" t="n"/>
-      <c r="F41" s="6" t="n"/>
+        <v>4.702677</v>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>56.220516</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>55.529352</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>14.822931</v>
+      </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1903,11 +2125,17 @@
         <v>44228</v>
       </c>
       <c r="C42" s="8" t="n">
-        <v>4.3974</v>
-      </c>
-      <c r="D42" s="8" t="n"/>
-      <c r="E42" s="8" t="n"/>
-      <c r="F42" s="8" t="n"/>
+        <v>4.397394</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>56.760047</v>
+      </c>
+      <c r="E42" s="8" t="n">
+        <v>55.336492</v>
+      </c>
+      <c r="F42" s="8" t="n">
+        <v>13.809624</v>
+      </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1939,11 +2167,17 @@
         <v>44256</v>
       </c>
       <c r="C43" s="6" t="n">
-        <v>3.8703</v>
-      </c>
-      <c r="D43" s="6" t="n"/>
-      <c r="E43" s="6" t="n"/>
-      <c r="F43" s="6" t="n"/>
+        <v>3.870291</v>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>57.284001</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>56.660104</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>13.022864</v>
+      </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -1975,11 +2209,17 @@
         <v>44287</v>
       </c>
       <c r="C44" s="8" t="n">
-        <v>4.6527</v>
-      </c>
-      <c r="D44" s="8" t="n"/>
-      <c r="E44" s="8" t="n"/>
-      <c r="F44" s="8" t="n"/>
+        <v>4.652681</v>
+      </c>
+      <c r="D44" s="8" t="n">
+        <v>59.053431</v>
+      </c>
+      <c r="E44" s="8" t="n">
+        <v>55.591673</v>
+      </c>
+      <c r="F44" s="8" t="n">
+        <v>13.712402</v>
+      </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2011,11 +2251,17 @@
         <v>44317</v>
       </c>
       <c r="C45" s="6" t="n">
-        <v>3.9939</v>
-      </c>
-      <c r="D45" s="6" t="n"/>
-      <c r="E45" s="6" t="n"/>
-      <c r="F45" s="6" t="n"/>
+        <v>3.993946</v>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>58.695716</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>55.538756</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>12.875162</v>
+      </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2047,11 +2293,17 @@
         <v>44348</v>
       </c>
       <c r="C46" s="8" t="n">
-        <v>4.0238</v>
-      </c>
-      <c r="D46" s="8" t="n"/>
-      <c r="E46" s="8" t="n"/>
-      <c r="F46" s="8" t="n"/>
+        <v>4.023772</v>
+      </c>
+      <c r="D46" s="8" t="n">
+        <v>58.480586</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>55.373765</v>
+      </c>
+      <c r="F46" s="8" t="n">
+        <v>12.362639</v>
+      </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2083,11 +2335,17 @@
         <v>44378</v>
       </c>
       <c r="C47" s="6" t="n">
-        <v>4.3822</v>
-      </c>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
+        <v>4.382247</v>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>59.914953</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>56.382507</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>13.231025</v>
+      </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2119,11 +2377,17 @@
         <v>44409</v>
       </c>
       <c r="C48" s="8" t="n">
-        <v>4.3263</v>
-      </c>
-      <c r="D48" s="8" t="n"/>
-      <c r="E48" s="8" t="n"/>
-      <c r="F48" s="8" t="n"/>
+        <v>4.326319</v>
+      </c>
+      <c r="D48" s="8" t="n">
+        <v>59.391912</v>
+      </c>
+      <c r="E48" s="8" t="n">
+        <v>56.355957</v>
+      </c>
+      <c r="F48" s="8" t="n">
+        <v>13.014263</v>
+      </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2155,11 +2419,17 @@
         <v>44440</v>
       </c>
       <c r="C49" s="6" t="n">
-        <v>4.185</v>
-      </c>
-      <c r="D49" s="6" t="n"/>
-      <c r="E49" s="6" t="n"/>
-      <c r="F49" s="6" t="n"/>
+        <v>4.184966</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <v>58.352771</v>
+      </c>
+      <c r="E49" s="6" t="n">
+        <v>56.17719</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>12.278231</v>
+      </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2191,11 +2461,17 @@
         <v>44470</v>
       </c>
       <c r="C50" s="8" t="n">
-        <v>3.9498</v>
-      </c>
-      <c r="D50" s="8" t="n"/>
-      <c r="E50" s="8" t="n"/>
-      <c r="F50" s="8" t="n"/>
+        <v>3.949786</v>
+      </c>
+      <c r="D50" s="8" t="n">
+        <v>59.443991</v>
+      </c>
+      <c r="E50" s="8" t="n">
+        <v>55.611833</v>
+      </c>
+      <c r="F50" s="8" t="n">
+        <v>11.072339</v>
+      </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2227,11 +2503,17 @@
         <v>44501</v>
       </c>
       <c r="C51" s="6" t="n">
-        <v>3.6649</v>
-      </c>
-      <c r="D51" s="6" t="n"/>
-      <c r="E51" s="6" t="n"/>
-      <c r="F51" s="6" t="n"/>
+        <v>3.664898</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <v>59.559287</v>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>55.638266</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>10.48903</v>
+      </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2263,11 +2545,17 @@
         <v>44531</v>
       </c>
       <c r="C52" s="8" t="n">
-        <v>3.5145</v>
-      </c>
-      <c r="D52" s="8" t="n"/>
-      <c r="E52" s="8" t="n"/>
-      <c r="F52" s="8" t="n"/>
+        <v>3.514471</v>
+      </c>
+      <c r="D52" s="8" t="n">
+        <v>59.513915</v>
+      </c>
+      <c r="E52" s="8" t="n">
+        <v>56.487632</v>
+      </c>
+      <c r="F52" s="8" t="n">
+        <v>10.006155</v>
+      </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2299,11 +2587,17 @@
         <v>44562</v>
       </c>
       <c r="C53" s="6" t="n">
-        <v>3.7069</v>
-      </c>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
+        <v>3.706941</v>
+      </c>
+      <c r="D53" s="6" t="n">
+        <v>58.334265</v>
+      </c>
+      <c r="E53" s="6" t="n">
+        <v>54.854561</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>9.096994</v>
+      </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2335,11 +2629,17 @@
         <v>44593</v>
       </c>
       <c r="C54" s="8" t="n">
-        <v>3.7412</v>
-      </c>
-      <c r="D54" s="8" t="n"/>
-      <c r="E54" s="8" t="n"/>
-      <c r="F54" s="8" t="n"/>
+        <v>3.741218</v>
+      </c>
+      <c r="D54" s="8" t="n">
+        <v>58.704869</v>
+      </c>
+      <c r="E54" s="8" t="n">
+        <v>54.617147</v>
+      </c>
+      <c r="F54" s="8" t="n">
+        <v>9.223545</v>
+      </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2371,11 +2671,17 @@
         <v>44621</v>
       </c>
       <c r="C55" s="6" t="n">
-        <v>2.9701</v>
-      </c>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
+        <v>2.970057</v>
+      </c>
+      <c r="D55" s="6" t="n">
+        <v>58.838103</v>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>55.785997</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>8.423329000000001</v>
+      </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2407,11 +2713,17 @@
         <v>44652</v>
       </c>
       <c r="C56" s="8" t="n">
-        <v>3.0341</v>
-      </c>
-      <c r="D56" s="8" t="n"/>
-      <c r="E56" s="8" t="n"/>
-      <c r="F56" s="8" t="n"/>
+        <v>3.034145</v>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>60.064497</v>
+      </c>
+      <c r="E56" s="8" t="n">
+        <v>55.531939</v>
+      </c>
+      <c r="F56" s="8" t="n">
+        <v>9.023562999999999</v>
+      </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2443,11 +2755,17 @@
         <v>44682</v>
       </c>
       <c r="C57" s="6" t="n">
-        <v>3.2705</v>
-      </c>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
+        <v>3.270451</v>
+      </c>
+      <c r="D57" s="6" t="n">
+        <v>59.606624</v>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>55.60542</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>8.478477</v>
+      </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2479,11 +2797,17 @@
         <v>44713</v>
       </c>
       <c r="C58" s="8" t="n">
-        <v>3.3487</v>
-      </c>
-      <c r="D58" s="8" t="n"/>
-      <c r="E58" s="8" t="n"/>
-      <c r="F58" s="8" t="n"/>
+        <v>3.34871</v>
+      </c>
+      <c r="D58" s="8" t="n">
+        <v>59.80334</v>
+      </c>
+      <c r="E58" s="8" t="n">
+        <v>55.842268</v>
+      </c>
+      <c r="F58" s="8" t="n">
+        <v>8.893288999999999</v>
+      </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2515,11 +2839,17 @@
         <v>44743</v>
       </c>
       <c r="C59" s="6" t="n">
-        <v>3.434</v>
-      </c>
-      <c r="D59" s="6" t="n"/>
-      <c r="E59" s="6" t="n"/>
-      <c r="F59" s="6" t="n"/>
+        <v>3.434004</v>
+      </c>
+      <c r="D59" s="6" t="n">
+        <v>60.006548</v>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>55.411656</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>8.254403999999999</v>
+      </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2551,11 +2881,17 @@
         <v>44774</v>
       </c>
       <c r="C60" s="8" t="n">
-        <v>3.5334</v>
-      </c>
-      <c r="D60" s="8" t="n"/>
-      <c r="E60" s="8" t="n"/>
-      <c r="F60" s="8" t="n"/>
+        <v>3.533439</v>
+      </c>
+      <c r="D60" s="8" t="n">
+        <v>59.998245</v>
+      </c>
+      <c r="E60" s="8" t="n">
+        <v>55.456146</v>
+      </c>
+      <c r="F60" s="8" t="n">
+        <v>7.889792</v>
+      </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2587,11 +2923,17 @@
         <v>44805</v>
       </c>
       <c r="C61" s="6" t="n">
-        <v>3.3362</v>
-      </c>
-      <c r="D61" s="6" t="n"/>
-      <c r="E61" s="6" t="n"/>
-      <c r="F61" s="6" t="n"/>
+        <v>3.336178</v>
+      </c>
+      <c r="D61" s="6" t="n">
+        <v>59.635154</v>
+      </c>
+      <c r="E61" s="6" t="n">
+        <v>55.580072</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>7.880164</v>
+      </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2623,11 +2965,17 @@
         <v>44835</v>
       </c>
       <c r="C62" s="8" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="D62" s="8" t="n"/>
-      <c r="E62" s="8" t="n"/>
-      <c r="F62" s="8" t="n"/>
+        <v>3.299988</v>
+      </c>
+      <c r="D62" s="8" t="n">
+        <v>60.696801</v>
+      </c>
+      <c r="E62" s="8" t="n">
+        <v>55.37724</v>
+      </c>
+      <c r="F62" s="8" t="n">
+        <v>7.468577</v>
+      </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2659,11 +3007,17 @@
         <v>44866</v>
       </c>
       <c r="C63" s="6" t="n">
-        <v>2.8468</v>
-      </c>
-      <c r="D63" s="6" t="n"/>
-      <c r="E63" s="6" t="n"/>
-      <c r="F63" s="6" t="n"/>
+        <v>2.846772</v>
+      </c>
+      <c r="D63" s="6" t="n">
+        <v>60.813189</v>
+      </c>
+      <c r="E63" s="6" t="n">
+        <v>55.166176</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>7.587039</v>
+      </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2695,11 +3049,17 @@
         <v>44896</v>
       </c>
       <c r="C64" s="8" t="n">
-        <v>2.7634</v>
-      </c>
-      <c r="D64" s="8" t="n"/>
-      <c r="E64" s="8" t="n"/>
-      <c r="F64" s="8" t="n"/>
+        <v>2.763351</v>
+      </c>
+      <c r="D64" s="8" t="n">
+        <v>59.692965</v>
+      </c>
+      <c r="E64" s="8" t="n">
+        <v>54.902761</v>
+      </c>
+      <c r="F64" s="8" t="n">
+        <v>7.257059</v>
+      </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2731,11 +3091,17 @@
         <v>44927</v>
       </c>
       <c r="C65" s="6" t="n">
-        <v>2.9997</v>
-      </c>
-      <c r="D65" s="6" t="n"/>
-      <c r="E65" s="6" t="n"/>
-      <c r="F65" s="6" t="n"/>
+        <v>2.999661</v>
+      </c>
+      <c r="D65" s="6" t="n">
+        <v>60.283485</v>
+      </c>
+      <c r="E65" s="6" t="n">
+        <v>54.815006</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>7.683689</v>
+      </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2767,11 +3133,17 @@
         <v>44958</v>
       </c>
       <c r="C66" s="8" t="n">
-        <v>2.7204</v>
-      </c>
-      <c r="D66" s="8" t="n"/>
-      <c r="E66" s="8" t="n"/>
-      <c r="F66" s="8" t="n"/>
+        <v>2.720432</v>
+      </c>
+      <c r="D66" s="8" t="n">
+        <v>60.183931</v>
+      </c>
+      <c r="E66" s="8" t="n">
+        <v>55.494593</v>
+      </c>
+      <c r="F66" s="8" t="n">
+        <v>7.379471</v>
+      </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2803,11 +3175,17 @@
         <v>44986</v>
       </c>
       <c r="C67" s="6" t="n">
-        <v>2.3925</v>
-      </c>
-      <c r="D67" s="6" t="n"/>
-      <c r="E67" s="6" t="n"/>
-      <c r="F67" s="6" t="n"/>
+        <v>2.392541</v>
+      </c>
+      <c r="D67" s="6" t="n">
+        <v>60.454729</v>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>54.98653</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>6.824846</v>
+      </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2839,11 +3217,17 @@
         <v>45017</v>
       </c>
       <c r="C68" s="8" t="n">
-        <v>2.8228</v>
-      </c>
-      <c r="D68" s="8" t="n"/>
-      <c r="E68" s="8" t="n"/>
-      <c r="F68" s="8" t="n"/>
+        <v>2.822799</v>
+      </c>
+      <c r="D68" s="8" t="n">
+        <v>60.356393</v>
+      </c>
+      <c r="E68" s="8" t="n">
+        <v>54.700335</v>
+      </c>
+      <c r="F68" s="8" t="n">
+        <v>8.396943</v>
+      </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2875,11 +3259,17 @@
         <v>45047</v>
       </c>
       <c r="C69" s="6" t="n">
-        <v>2.9311</v>
-      </c>
-      <c r="D69" s="6" t="n"/>
-      <c r="E69" s="6" t="n"/>
-      <c r="F69" s="6" t="n"/>
+        <v>2.931125</v>
+      </c>
+      <c r="D69" s="6" t="n">
+        <v>60.01101</v>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>55.169572</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>8.090506</v>
+      </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2911,11 +3301,17 @@
         <v>45078</v>
       </c>
       <c r="C70" s="8" t="n">
-        <v>2.652</v>
-      </c>
-      <c r="D70" s="8" t="n"/>
-      <c r="E70" s="8" t="n"/>
-      <c r="F70" s="8" t="n"/>
+        <v>2.652033</v>
+      </c>
+      <c r="D70" s="8" t="n">
+        <v>60.115145</v>
+      </c>
+      <c r="E70" s="8" t="n">
+        <v>55.486488</v>
+      </c>
+      <c r="F70" s="8" t="n">
+        <v>7.860973</v>
+      </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2947,11 +3343,17 @@
         <v>45108</v>
       </c>
       <c r="C71" s="6" t="n">
-        <v>3.1299</v>
-      </c>
-      <c r="D71" s="6" t="n"/>
-      <c r="E71" s="6" t="n"/>
-      <c r="F71" s="6" t="n"/>
+        <v>3.12987</v>
+      </c>
+      <c r="D71" s="6" t="n">
+        <v>60.87252</v>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>55.713385</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>8.064282</v>
+      </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -2983,11 +3385,17 @@
         <v>45139</v>
       </c>
       <c r="C72" s="8" t="n">
-        <v>2.9553</v>
-      </c>
-      <c r="D72" s="8" t="n"/>
-      <c r="E72" s="8" t="n"/>
-      <c r="F72" s="8" t="n"/>
+        <v>2.955346</v>
+      </c>
+      <c r="D72" s="8" t="n">
+        <v>60.533479</v>
+      </c>
+      <c r="E72" s="8" t="n">
+        <v>55.248993</v>
+      </c>
+      <c r="F72" s="8" t="n">
+        <v>7.908474</v>
+      </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3019,11 +3427,17 @@
         <v>45170</v>
       </c>
       <c r="C73" s="6" t="n">
-        <v>2.8774</v>
-      </c>
-      <c r="D73" s="6" t="n"/>
-      <c r="E73" s="6" t="n"/>
-      <c r="F73" s="6" t="n"/>
+        <v>2.877421</v>
+      </c>
+      <c r="D73" s="6" t="n">
+        <v>60.357718</v>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>54.303345</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>8.170244</v>
+      </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3055,11 +3469,17 @@
         <v>45200</v>
       </c>
       <c r="C74" s="8" t="n">
-        <v>2.746</v>
-      </c>
-      <c r="D74" s="8" t="n"/>
-      <c r="E74" s="8" t="n"/>
-      <c r="F74" s="8" t="n"/>
+        <v>2.745996</v>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>60.459268</v>
+      </c>
+      <c r="E74" s="8" t="n">
+        <v>55.40583</v>
+      </c>
+      <c r="F74" s="8" t="n">
+        <v>7.863639</v>
+      </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3091,11 +3511,17 @@
         <v>45231</v>
       </c>
       <c r="C75" s="6" t="n">
-        <v>2.7127</v>
-      </c>
-      <c r="D75" s="6" t="n"/>
-      <c r="E75" s="6" t="n"/>
-      <c r="F75" s="6" t="n"/>
+        <v>2.712708</v>
+      </c>
+      <c r="D75" s="6" t="n">
+        <v>60.959679</v>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>54.730362</v>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>8.209669</v>
+      </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3127,11 +3553,17 @@
         <v>45261</v>
       </c>
       <c r="C76" s="8" t="n">
-        <v>2.6138</v>
-      </c>
-      <c r="D76" s="8" t="n"/>
-      <c r="E76" s="8" t="n"/>
-      <c r="F76" s="8" t="n"/>
+        <v>2.61376</v>
+      </c>
+      <c r="D76" s="8" t="n">
+        <v>59.866851</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <v>53.626856</v>
+      </c>
+      <c r="F76" s="8" t="n">
+        <v>7.632108</v>
+      </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3163,11 +3595,17 @@
         <v>45292</v>
       </c>
       <c r="C77" s="6" t="n">
-        <v>2.853</v>
-      </c>
-      <c r="D77" s="6" t="n"/>
-      <c r="E77" s="6" t="n"/>
-      <c r="F77" s="6" t="n"/>
+        <v>2.853024</v>
+      </c>
+      <c r="D77" s="6" t="n">
+        <v>59.772911</v>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>54.11355</v>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>7.078092</v>
+      </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3199,11 +3637,17 @@
         <v>45323</v>
       </c>
       <c r="C78" s="8" t="n">
-        <v>2.454</v>
-      </c>
-      <c r="D78" s="8" t="n"/>
-      <c r="E78" s="8" t="n"/>
-      <c r="F78" s="8" t="n"/>
+        <v>2.454003</v>
+      </c>
+      <c r="D78" s="8" t="n">
+        <v>60.17459</v>
+      </c>
+      <c r="E78" s="8" t="n">
+        <v>54.467561</v>
+      </c>
+      <c r="F78" s="8" t="n">
+        <v>6.467305</v>
+      </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3235,11 +3679,17 @@
         <v>45352</v>
       </c>
       <c r="C79" s="6" t="n">
-        <v>2.2821</v>
-      </c>
-      <c r="D79" s="6" t="n"/>
-      <c r="E79" s="6" t="n"/>
-      <c r="F79" s="6" t="n"/>
+        <v>2.282067</v>
+      </c>
+      <c r="D79" s="6" t="n">
+        <v>60.169544</v>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>54.303549</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>6.519986</v>
+      </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3271,11 +3721,17 @@
         <v>45383</v>
       </c>
       <c r="C80" s="8" t="n">
-        <v>2.6107</v>
-      </c>
-      <c r="D80" s="8" t="n"/>
-      <c r="E80" s="8" t="n"/>
-      <c r="F80" s="8" t="n"/>
+        <v>2.610737</v>
+      </c>
+      <c r="D80" s="8" t="n">
+        <v>60.477015</v>
+      </c>
+      <c r="E80" s="8" t="n">
+        <v>54.555735</v>
+      </c>
+      <c r="F80" s="8" t="n">
+        <v>7.735678</v>
+      </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3307,11 +3763,17 @@
         <v>45413</v>
       </c>
       <c r="C81" s="6" t="n">
-        <v>2.6218</v>
-      </c>
-      <c r="D81" s="6" t="n"/>
-      <c r="E81" s="6" t="n"/>
-      <c r="F81" s="6" t="n"/>
+        <v>2.621775</v>
+      </c>
+      <c r="D81" s="6" t="n">
+        <v>60.535248</v>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>54.448946</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>7.425446</v>
+      </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3343,11 +3805,17 @@
         <v>45444</v>
       </c>
       <c r="C82" s="8" t="n">
-        <v>2.775</v>
-      </c>
-      <c r="D82" s="8" t="n"/>
-      <c r="E82" s="8" t="n"/>
-      <c r="F82" s="8" t="n"/>
+        <v>2.775024</v>
+      </c>
+      <c r="D82" s="8" t="n">
+        <v>59.836994</v>
+      </c>
+      <c r="E82" s="8" t="n">
+        <v>53.838213</v>
+      </c>
+      <c r="F82" s="8" t="n">
+        <v>7.501859</v>
+      </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3379,11 +3847,17 @@
         <v>45474</v>
       </c>
       <c r="C83" s="6" t="n">
-        <v>2.9274</v>
-      </c>
-      <c r="D83" s="6" t="n"/>
-      <c r="E83" s="6" t="n"/>
-      <c r="F83" s="6" t="n"/>
+        <v>2.927401</v>
+      </c>
+      <c r="D83" s="6" t="n">
+        <v>61.041278</v>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>54.516061</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>8.052058000000001</v>
+      </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3415,11 +3889,17 @@
         <v>45505</v>
       </c>
       <c r="C84" s="8" t="n">
-        <v>3.0374</v>
-      </c>
-      <c r="D84" s="8" t="n"/>
-      <c r="E84" s="8" t="n"/>
-      <c r="F84" s="8" t="n"/>
+        <v>3.037372</v>
+      </c>
+      <c r="D84" s="8" t="n">
+        <v>60.192452</v>
+      </c>
+      <c r="E84" s="8" t="n">
+        <v>54.303891</v>
+      </c>
+      <c r="F84" s="8" t="n">
+        <v>7.99311</v>
+      </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3451,11 +3931,17 @@
         <v>45536</v>
       </c>
       <c r="C85" s="6" t="n">
-        <v>2.9225</v>
-      </c>
-      <c r="D85" s="6" t="n"/>
-      <c r="E85" s="6" t="n"/>
-      <c r="F85" s="6" t="n"/>
+        <v>2.922514</v>
+      </c>
+      <c r="D85" s="6" t="n">
+        <v>59.974784</v>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>54.240017</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>8.171984</v>
+      </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3487,11 +3973,17 @@
         <v>45566</v>
       </c>
       <c r="C86" s="8" t="n">
-        <v>2.5002</v>
-      </c>
-      <c r="D86" s="8" t="n"/>
-      <c r="E86" s="8" t="n"/>
-      <c r="F86" s="8" t="n"/>
+        <v>2.500182</v>
+      </c>
+      <c r="D86" s="8" t="n">
+        <v>60.230403</v>
+      </c>
+      <c r="E86" s="8" t="n">
+        <v>54.131321</v>
+      </c>
+      <c r="F86" s="8" t="n">
+        <v>9.379963</v>
+      </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3523,11 +4015,17 @@
         <v>45597</v>
       </c>
       <c r="C87" s="6" t="n">
-        <v>2.6388</v>
-      </c>
-      <c r="D87" s="6" t="n"/>
-      <c r="E87" s="6" t="n"/>
-      <c r="F87" s="6" t="n"/>
+        <v>2.638833</v>
+      </c>
+      <c r="D87" s="6" t="n">
+        <v>60.045171</v>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>54.630964</v>
+      </c>
+      <c r="F87" s="6" t="n">
+        <v>8.855615</v>
+      </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3559,11 +4057,17 @@
         <v>45627</v>
       </c>
       <c r="C88" s="8" t="n">
-        <v>2.4323</v>
-      </c>
-      <c r="D88" s="8" t="n"/>
-      <c r="E88" s="8" t="n"/>
-      <c r="F88" s="8" t="n"/>
+        <v>2.432341</v>
+      </c>
+      <c r="D88" s="8" t="n">
+        <v>59.320476</v>
+      </c>
+      <c r="E88" s="8" t="n">
+        <v>53.651825</v>
+      </c>
+      <c r="F88" s="8" t="n">
+        <v>6.862197</v>
+      </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3595,11 +4099,17 @@
         <v>45658</v>
       </c>
       <c r="C89" s="6" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="D89" s="6" t="n"/>
-      <c r="E89" s="6" t="n"/>
-      <c r="F89" s="6" t="n"/>
+        <v>2.699951</v>
+      </c>
+      <c r="D89" s="6" t="n">
+        <v>59.36401</v>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>54.136601</v>
+      </c>
+      <c r="F89" s="6" t="n">
+        <v>6.94748</v>
+      </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3631,11 +4141,17 @@
         <v>45689</v>
       </c>
       <c r="C90" s="8" t="n">
-        <v>2.5114</v>
-      </c>
-      <c r="D90" s="8" t="n"/>
-      <c r="E90" s="8" t="n"/>
-      <c r="F90" s="8" t="n"/>
+        <v>2.51142</v>
+      </c>
+      <c r="D90" s="8" t="n">
+        <v>58.714231</v>
+      </c>
+      <c r="E90" s="8" t="n">
+        <v>54.510303</v>
+      </c>
+      <c r="F90" s="8" t="n">
+        <v>6.259252</v>
+      </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3667,11 +4183,17 @@
         <v>45717</v>
       </c>
       <c r="C91" s="6" t="n">
-        <v>2.2222</v>
-      </c>
-      <c r="D91" s="6" t="n"/>
-      <c r="E91" s="6" t="n"/>
-      <c r="F91" s="6" t="n"/>
+        <v>2.222196</v>
+      </c>
+      <c r="D91" s="6" t="n">
+        <v>59.343805</v>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>54.337696</v>
+      </c>
+      <c r="F91" s="6" t="n">
+        <v>6.601645</v>
+      </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3703,11 +4225,17 @@
         <v>45748</v>
       </c>
       <c r="C92" s="8" t="n">
-        <v>2.5391</v>
-      </c>
-      <c r="D92" s="8" t="n"/>
-      <c r="E92" s="8" t="n"/>
-      <c r="F92" s="8" t="n"/>
+        <v>2.539106</v>
+      </c>
+      <c r="D92" s="8" t="n">
+        <v>59.369192</v>
+      </c>
+      <c r="E92" s="8" t="n">
+        <v>54.671184</v>
+      </c>
+      <c r="F92" s="8" t="n">
+        <v>7.146182</v>
+      </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3739,11 +4267,17 @@
         <v>45778</v>
       </c>
       <c r="C93" s="6" t="n">
-        <v>2.7463</v>
-      </c>
-      <c r="D93" s="6" t="n"/>
-      <c r="E93" s="6" t="n"/>
-      <c r="F93" s="6" t="n"/>
+        <v>2.746314</v>
+      </c>
+      <c r="D93" s="6" t="n">
+        <v>59.451546</v>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>54.920523</v>
+      </c>
+      <c r="F93" s="6" t="n">
+        <v>7.094072</v>
+      </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3775,11 +4309,17 @@
         <v>45809</v>
       </c>
       <c r="C94" s="8" t="n">
-        <v>2.6871</v>
-      </c>
-      <c r="D94" s="8" t="n"/>
-      <c r="E94" s="8" t="n"/>
-      <c r="F94" s="8" t="n"/>
+        <v>2.687124</v>
+      </c>
+      <c r="D94" s="8" t="n">
+        <v>59.797354</v>
+      </c>
+      <c r="E94" s="8" t="n">
+        <v>54.768222</v>
+      </c>
+      <c r="F94" s="8" t="n">
+        <v>7.354796</v>
+      </c>
       <c r="G94" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3811,11 +4351,17 @@
         <v>45839</v>
       </c>
       <c r="C95" s="6" t="n">
-        <v>2.7728</v>
-      </c>
-      <c r="D95" s="6" t="n"/>
-      <c r="E95" s="6" t="n"/>
-      <c r="F95" s="6" t="n"/>
+        <v>2.772825</v>
+      </c>
+      <c r="D95" s="6" t="n">
+        <v>60.176973</v>
+      </c>
+      <c r="E95" s="6" t="n">
+        <v>56.117157</v>
+      </c>
+      <c r="F95" s="6" t="n">
+        <v>7.34019</v>
+      </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3847,11 +4393,17 @@
         <v>45870</v>
       </c>
       <c r="C96" s="8" t="n">
-        <v>2.9322</v>
-      </c>
-      <c r="D96" s="8" t="n"/>
-      <c r="E96" s="8" t="n"/>
-      <c r="F96" s="8" t="n"/>
+        <v>2.932245</v>
+      </c>
+      <c r="D96" s="8" t="n">
+        <v>58.824828</v>
+      </c>
+      <c r="E96" s="8" t="n">
+        <v>54.825008</v>
+      </c>
+      <c r="F96" s="8" t="n">
+        <v>7.053359</v>
+      </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3883,11 +4435,17 @@
         <v>45901</v>
       </c>
       <c r="C97" s="6" t="n">
-        <v>2.9789</v>
-      </c>
-      <c r="D97" s="6" t="n"/>
-      <c r="E97" s="6" t="n"/>
-      <c r="F97" s="6" t="n"/>
+        <v>2.978907</v>
+      </c>
+      <c r="D97" s="6" t="n">
+        <v>59.568499</v>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v>54.879891</v>
+      </c>
+      <c r="F97" s="6" t="n">
+        <v>7.278606</v>
+      </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3919,11 +4477,17 @@
         <v>45931</v>
       </c>
       <c r="C98" s="8" t="n">
-        <v>2.6085</v>
-      </c>
-      <c r="D98" s="8" t="n"/>
-      <c r="E98" s="8" t="n"/>
-      <c r="F98" s="8" t="n"/>
+        <v>2.608456</v>
+      </c>
+      <c r="D98" s="8" t="n">
+        <v>59.912373</v>
+      </c>
+      <c r="E98" s="8" t="n">
+        <v>55.655124</v>
+      </c>
+      <c r="F98" s="8" t="n">
+        <v>7.528537</v>
+      </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3955,11 +4519,17 @@
         <v>45962</v>
       </c>
       <c r="C99" s="6" t="n">
-        <v>2.6636</v>
-      </c>
-      <c r="D99" s="6" t="n"/>
-      <c r="E99" s="6" t="n"/>
-      <c r="F99" s="6" t="n"/>
+        <v>2.663619</v>
+      </c>
+      <c r="D99" s="6" t="n">
+        <v>58.954439</v>
+      </c>
+      <c r="E99" s="6" t="n">
+        <v>54.793253</v>
+      </c>
+      <c r="F99" s="6" t="n">
+        <v>7.189759</v>
+      </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -3991,11 +4561,17 @@
         <v>45992</v>
       </c>
       <c r="C100" s="8" t="n">
-        <v>2.3889</v>
-      </c>
-      <c r="D100" s="8" t="n"/>
-      <c r="E100" s="8" t="n"/>
-      <c r="F100" s="8" t="n"/>
+        <v>2.388894</v>
+      </c>
+      <c r="D100" s="8" t="n">
+        <v>59.096571</v>
+      </c>
+      <c r="E100" s="8" t="n">
+        <v>54.636116</v>
+      </c>
+      <c r="F100" s="8" t="n">
+        <v>6.205645</v>
+      </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4027,11 +4603,17 @@
         <v>46023</v>
       </c>
       <c r="C101" s="6" t="n">
-        <v>2.7033</v>
-      </c>
-      <c r="D101" s="6" t="n"/>
-      <c r="E101" s="6" t="n"/>
-      <c r="F101" s="6" t="n"/>
+        <v>2.703262</v>
+      </c>
+      <c r="D101" s="6" t="n">
+        <v>58.504316</v>
+      </c>
+      <c r="E101" s="6" t="n">
+        <v>54.861145</v>
+      </c>
+      <c r="F101" s="6" t="n">
+        <v>6.114657</v>
+      </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4063,11 +4645,17 @@
         <v>46054</v>
       </c>
       <c r="C102" s="8" t="n">
-        <v>2.5862</v>
-      </c>
-      <c r="D102" s="8" t="n"/>
-      <c r="E102" s="8" t="n"/>
-      <c r="F102" s="8" t="n"/>
+        <v>2.586177</v>
+      </c>
+      <c r="D102" s="8" t="n">
+        <v>59.010645</v>
+      </c>
+      <c r="E102" s="8" t="n">
+        <v>54.764186</v>
+      </c>
+      <c r="F102" s="8" t="n">
+        <v>6.983543</v>
+      </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4099,11 +4687,17 @@
         <v>46082</v>
       </c>
       <c r="C103" s="6" t="n">
-        <v>2.4232</v>
-      </c>
-      <c r="D103" s="6" t="n"/>
-      <c r="E103" s="6" t="n"/>
-      <c r="F103" s="6" t="n"/>
+        <v>2.423162</v>
+      </c>
+      <c r="D103" s="6" t="n">
+        <v>58.581471</v>
+      </c>
+      <c r="E103" s="6" t="n">
+        <v>54.847369</v>
+      </c>
+      <c r="F103" s="6" t="n">
+        <v>6.721879</v>
+      </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4135,11 +4729,17 @@
         <v>46113</v>
       </c>
       <c r="C104" s="8" t="n">
-        <v>2.4558</v>
-      </c>
-      <c r="D104" s="8" t="n"/>
-      <c r="E104" s="8" t="n"/>
-      <c r="F104" s="8" t="n"/>
+        <v>2.455787</v>
+      </c>
+      <c r="D104" s="8" t="n">
+        <v>59.134706</v>
+      </c>
+      <c r="E104" s="8" t="n">
+        <v>55.180276</v>
+      </c>
+      <c r="F104" s="8" t="n">
+        <v>7.098691</v>
+      </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4171,11 +4771,17 @@
         <v>46143</v>
       </c>
       <c r="C105" s="6" t="n">
-        <v>2.7619</v>
-      </c>
-      <c r="D105" s="6" t="n"/>
-      <c r="E105" s="6" t="n"/>
-      <c r="F105" s="6" t="n"/>
+        <v>2.761933</v>
+      </c>
+      <c r="D105" s="6" t="n">
+        <v>59.092093</v>
+      </c>
+      <c r="E105" s="6" t="n">
+        <v>55.225275</v>
+      </c>
+      <c r="F105" s="6" t="n">
+        <v>6.976081</v>
+      </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4207,11 +4813,17 @@
         <v>46174</v>
       </c>
       <c r="C106" s="8" t="n">
-        <v>2.8985</v>
-      </c>
-      <c r="D106" s="8" t="n"/>
-      <c r="E106" s="8" t="n"/>
-      <c r="F106" s="8" t="n"/>
+        <v>2.898523</v>
+      </c>
+      <c r="D106" s="8" t="n">
+        <v>58.83743</v>
+      </c>
+      <c r="E106" s="8" t="n">
+        <v>55.019889</v>
+      </c>
+      <c r="F106" s="8" t="n">
+        <v>6.550443</v>
+      </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4326,8 +4938,12 @@
       <c r="B5" s="5" t="n">
         <v>43101</v>
       </c>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="11" t="n"/>
+      <c r="C5" s="10" t="n">
+        <v>52.253036</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>52253036</v>
+      </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4422,8 +5038,12 @@
       <c r="B8" s="5" t="n">
         <v>43191</v>
       </c>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="13" t="n"/>
+      <c r="C8" s="12" t="n">
+        <v>53.205163</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>53205163</v>
+      </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4518,8 +5138,12 @@
       <c r="B11" s="5" t="n">
         <v>43282</v>
       </c>
-      <c r="C11" s="10" t="n"/>
-      <c r="D11" s="11" t="n"/>
+      <c r="C11" s="10" t="n">
+        <v>53.483093</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>53483093</v>
+      </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4614,8 +5238,12 @@
       <c r="B14" s="5" t="n">
         <v>43374</v>
       </c>
-      <c r="C14" s="12" t="n"/>
-      <c r="D14" s="13" t="n"/>
+      <c r="C14" s="12" t="n">
+        <v>53.705872</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>53705872</v>
+      </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4710,8 +5338,12 @@
       <c r="B17" s="5" t="n">
         <v>43466</v>
       </c>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="11" t="n"/>
+      <c r="C17" s="10" t="n">
+        <v>53.714758</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>53714758</v>
+      </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4806,8 +5438,12 @@
       <c r="B20" s="5" t="n">
         <v>43556</v>
       </c>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="13" t="n"/>
+      <c r="C20" s="12" t="n">
+        <v>54.549769</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>54549769</v>
+      </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4902,8 +5538,12 @@
       <c r="B23" s="5" t="n">
         <v>43647</v>
       </c>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="11" t="n"/>
+      <c r="C23" s="10" t="n">
+        <v>54.848407</v>
+      </c>
+      <c r="D23" s="11" t="n">
+        <v>54848407</v>
+      </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -4998,8 +5638,12 @@
       <c r="B26" s="5" t="n">
         <v>43739</v>
       </c>
-      <c r="C26" s="12" t="n"/>
-      <c r="D26" s="13" t="n"/>
+      <c r="C26" s="12" t="n">
+        <v>55.345261</v>
+      </c>
+      <c r="D26" s="13" t="n">
+        <v>55345261</v>
+      </c>
       <c r="E26" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5094,8 +5738,12 @@
       <c r="B29" s="5" t="n">
         <v>43831</v>
       </c>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="11" t="n"/>
+      <c r="C29" s="10" t="n">
+        <v>55.05845</v>
+      </c>
+      <c r="D29" s="11" t="n">
+        <v>55058450</v>
+      </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5190,8 +5838,12 @@
       <c r="B32" s="5" t="n">
         <v>43922</v>
       </c>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="13" t="n"/>
+      <c r="C32" s="12" t="n">
+        <v>44.715068</v>
+      </c>
+      <c r="D32" s="13" t="n">
+        <v>44715067.666667</v>
+      </c>
       <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5286,8 +5938,12 @@
       <c r="B35" s="5" t="n">
         <v>44013</v>
       </c>
-      <c r="C35" s="10" t="n"/>
-      <c r="D35" s="11" t="n"/>
+      <c r="C35" s="10" t="n">
+        <v>50.810713</v>
+      </c>
+      <c r="D35" s="11" t="n">
+        <v>50810713</v>
+      </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5382,8 +6038,12 @@
       <c r="B38" s="5" t="n">
         <v>44105</v>
       </c>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="13" t="n"/>
+      <c r="C38" s="12" t="n">
+        <v>53.124071</v>
+      </c>
+      <c r="D38" s="13" t="n">
+        <v>53124071</v>
+      </c>
       <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5478,8 +6138,12 @@
       <c r="B41" s="5" t="n">
         <v>44197</v>
       </c>
-      <c r="C41" s="10" t="n"/>
-      <c r="D41" s="11" t="n"/>
+      <c r="C41" s="10" t="n">
+        <v>52.97327</v>
+      </c>
+      <c r="D41" s="11" t="n">
+        <v>52973270</v>
+      </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5574,8 +6238,12 @@
       <c r="B44" s="5" t="n">
         <v>44287</v>
       </c>
-      <c r="C44" s="12" t="n"/>
-      <c r="D44" s="13" t="n"/>
+      <c r="C44" s="12" t="n">
+        <v>55.242748</v>
+      </c>
+      <c r="D44" s="13" t="n">
+        <v>55242748</v>
+      </c>
       <c r="E44" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5670,8 +6338,12 @@
       <c r="B47" s="5" t="n">
         <v>44378</v>
       </c>
-      <c r="C47" s="10" t="n"/>
-      <c r="D47" s="11" t="n"/>
+      <c r="C47" s="10" t="n">
+        <v>55.83623</v>
+      </c>
+      <c r="D47" s="11" t="n">
+        <v>55836230</v>
+      </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5766,8 +6438,12 @@
       <c r="B50" s="5" t="n">
         <v>44470</v>
       </c>
-      <c r="C50" s="12" t="n"/>
-      <c r="D50" s="13" t="n"/>
+      <c r="C50" s="12" t="n">
+        <v>56.611211</v>
+      </c>
+      <c r="D50" s="13" t="n">
+        <v>56611211</v>
+      </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5862,8 +6538,12 @@
       <c r="B53" s="5" t="n">
         <v>44562</v>
       </c>
-      <c r="C53" s="10" t="n"/>
-      <c r="D53" s="11" t="n"/>
+      <c r="C53" s="10" t="n">
+        <v>56.079123</v>
+      </c>
+      <c r="D53" s="11" t="n">
+        <v>56079123</v>
+      </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -5958,8 +6638,12 @@
       <c r="B56" s="5" t="n">
         <v>44652</v>
       </c>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="13" t="n"/>
+      <c r="C56" s="12" t="n">
+        <v>57.420677</v>
+      </c>
+      <c r="D56" s="13" t="n">
+        <v>57420677</v>
+      </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6054,8 +6738,12 @@
       <c r="B59" s="5" t="n">
         <v>44743</v>
       </c>
-      <c r="C59" s="10" t="n"/>
-      <c r="D59" s="11" t="n"/>
+      <c r="C59" s="10" t="n">
+        <v>57.440441</v>
+      </c>
+      <c r="D59" s="11" t="n">
+        <v>57440441</v>
+      </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6150,8 +6838,12 @@
       <c r="B62" s="5" t="n">
         <v>44835</v>
       </c>
-      <c r="C62" s="12" t="n"/>
-      <c r="D62" s="13" t="n"/>
+      <c r="C62" s="12" t="n">
+        <v>58.349353</v>
+      </c>
+      <c r="D62" s="13" t="n">
+        <v>58349353</v>
+      </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6246,8 +6938,12 @@
       <c r="B65" s="5" t="n">
         <v>44927</v>
       </c>
-      <c r="C65" s="10" t="n"/>
-      <c r="D65" s="11" t="n"/>
+      <c r="C65" s="10" t="n">
+        <v>58.492126</v>
+      </c>
+      <c r="D65" s="11" t="n">
+        <v>58492126</v>
+      </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6342,8 +7038,12 @@
       <c r="B68" s="5" t="n">
         <v>45017</v>
       </c>
-      <c r="C68" s="12" t="n"/>
-      <c r="D68" s="13" t="n"/>
+      <c r="C68" s="12" t="n">
+        <v>58.52199</v>
+      </c>
+      <c r="D68" s="13" t="n">
+        <v>58521990</v>
+      </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6438,8 +7138,12 @@
       <c r="B71" s="5" t="n">
         <v>45108</v>
       </c>
-      <c r="C71" s="10" t="n"/>
-      <c r="D71" s="11" t="n"/>
+      <c r="C71" s="10" t="n">
+        <v>59.167472</v>
+      </c>
+      <c r="D71" s="11" t="n">
+        <v>59167472</v>
+      </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6534,8 +7238,12 @@
       <c r="B74" s="5" t="n">
         <v>45200</v>
       </c>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="13" t="n"/>
+      <c r="C74" s="12" t="n">
+        <v>59.403947</v>
+      </c>
+      <c r="D74" s="13" t="n">
+        <v>59403947</v>
+      </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6630,8 +7338,12 @@
       <c r="B77" s="5" t="n">
         <v>45292</v>
       </c>
-      <c r="C77" s="10" t="n"/>
-      <c r="D77" s="11" t="n"/>
+      <c r="C77" s="10" t="n">
+        <v>59.120905</v>
+      </c>
+      <c r="D77" s="11" t="n">
+        <v>59120905</v>
+      </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6726,8 +7438,12 @@
       <c r="B80" s="5" t="n">
         <v>45383</v>
       </c>
-      <c r="C80" s="12" t="n"/>
-      <c r="D80" s="13" t="n"/>
+      <c r="C80" s="12" t="n">
+        <v>59.327161</v>
+      </c>
+      <c r="D80" s="13" t="n">
+        <v>59327161</v>
+      </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6822,8 +7538,12 @@
       <c r="B83" s="5" t="n">
         <v>45474</v>
       </c>
-      <c r="C83" s="10" t="n"/>
-      <c r="D83" s="11" t="n"/>
+      <c r="C83" s="10" t="n">
+        <v>59.528249</v>
+      </c>
+      <c r="D83" s="11" t="n">
+        <v>59528249</v>
+      </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -6918,8 +7638,12 @@
       <c r="B86" s="5" t="n">
         <v>45566</v>
       </c>
-      <c r="C86" s="12" t="n"/>
-      <c r="D86" s="13" t="n"/>
+      <c r="C86" s="12" t="n">
+        <v>59.487546</v>
+      </c>
+      <c r="D86" s="13" t="n">
+        <v>59487546</v>
+      </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -7014,8 +7738,12 @@
       <c r="B89" s="5" t="n">
         <v>45658</v>
       </c>
-      <c r="C89" s="10" t="n"/>
-      <c r="D89" s="11" t="n"/>
+      <c r="C89" s="10" t="n">
+        <v>59.001009</v>
+      </c>
+      <c r="D89" s="11" t="n">
+        <v>59001009</v>
+      </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -7110,8 +7838,12 @@
       <c r="B92" s="5" t="n">
         <v>45748</v>
       </c>
-      <c r="C92" s="12" t="n"/>
-      <c r="D92" s="13" t="n"/>
+      <c r="C92" s="12" t="n">
+        <v>59.44076</v>
+      </c>
+      <c r="D92" s="13" t="n">
+        <v>59440760</v>
+      </c>
       <c r="E92" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -7206,8 +7938,12 @@
       <c r="B95" s="5" t="n">
         <v>45839</v>
       </c>
-      <c r="C95" s="10" t="n"/>
-      <c r="D95" s="11" t="n"/>
+      <c r="C95" s="10" t="n">
+        <v>59.533449</v>
+      </c>
+      <c r="D95" s="11" t="n">
+        <v>59533449</v>
+      </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -7302,8 +8038,12 @@
       <c r="B98" s="5" t="n">
         <v>45931</v>
       </c>
-      <c r="C98" s="12" t="n"/>
-      <c r="D98" s="13" t="n"/>
+      <c r="C98" s="12" t="n">
+        <v>59.785854</v>
+      </c>
+      <c r="D98" s="13" t="n">
+        <v>59785854</v>
+      </c>
       <c r="E98" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -7398,8 +8138,12 @@
       <c r="B101" s="5" t="n">
         <v>46023</v>
       </c>
-      <c r="C101" s="10" t="n"/>
-      <c r="D101" s="11" t="n"/>
+      <c r="C101" s="10" t="n">
+        <v>59.55266</v>
+      </c>
+      <c r="D101" s="11" t="n">
+        <v>59552660</v>
+      </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
           <t>Definitivo</t>
@@ -7494,8 +8238,12 @@
       <c r="B104" s="5" t="n">
         <v>46113</v>
       </c>
-      <c r="C104" s="12" t="n"/>
-      <c r="D104" s="13" t="n"/>
+      <c r="C104" s="12" t="n">
+        <v>60.040094</v>
+      </c>
+      <c r="D104" s="13" t="n">
+        <v>60040094</v>
+      </c>
       <c r="E104" s="9" t="inlineStr">
         <is>
           <t>Definitivo</t>

</xml_diff>

<commit_message>
feat(inpp): integra el Índice Nacional de Precios Productor en el dashboard.
Añade el conector scripts/sources/inegi_inpp.py, que consulta niveles,
variaciones mensuales/anuales/acumuladas y componentes del BIE de INEGI.
Actualiza build_data.py y lib_data.py para soportar nuevos indicadores
 desde el perfil, integra INPP en la configuración frontend/backend,
actualiza el calendario, el boletín oficial, las notas, los tests y
genera los archivos Excel individuales y consolidado.

Datos regenerados y validados:
- build_data, build_excel, build_calendar, validate y pytest pasan.
- 0 errores críticos, 113 tests passed.

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/downloads/indicadores/DESOCUP/DESOCUP_datos.xlsx
+++ b/downloads/indicadores/DESOCUP/DESOCUP_datos.xlsx
@@ -480,7 +480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -505,7 +505,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: INEGI — Encuesta Nacional de Ocupación y Empleo (ENOE/ENOEN) · Frecuencia: Mensual · Unidad: porcentaje · Boletín: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf · Fecha de publicación: 24 de julio de 2026</t>
+          <t>Fuente: INEGI — Encuesta Nacional de Ocupación y Empleo (ENOE/ENOEN) · Frecuencia: Mensual · Unidad: porcentaje · Boletín: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf · Fecha de publicación: 27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -594,12 +594,12 @@
       </c>
       <c r="I5" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -636,12 +636,12 @@
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J6" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -678,12 +678,12 @@
       </c>
       <c r="I7" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -720,12 +720,12 @@
       </c>
       <c r="I8" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J8" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="I9" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -804,12 +804,12 @@
       </c>
       <c r="I10" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J10" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -846,12 +846,12 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J11" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -888,12 +888,12 @@
       </c>
       <c r="I12" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J12" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -930,12 +930,12 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J13" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -972,12 +972,12 @@
       </c>
       <c r="I14" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J14" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1014,12 +1014,12 @@
       </c>
       <c r="I15" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="I16" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J16" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1098,12 +1098,12 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1140,12 @@
       </c>
       <c r="I18" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J18" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1182,12 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1224,12 +1224,12 @@
       </c>
       <c r="I20" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1266,12 +1266,12 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1308,12 +1308,12 @@
       </c>
       <c r="I22" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J22" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1350,12 +1350,12 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1392,12 +1392,12 @@
       </c>
       <c r="I24" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J24" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1434,12 +1434,12 @@
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J25" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1476,12 @@
       </c>
       <c r="I26" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J26" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1518,12 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J27" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1560,12 +1560,12 @@
       </c>
       <c r="I28" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J28" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1602,12 +1602,12 @@
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1644,12 +1644,12 @@
       </c>
       <c r="I30" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J30" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1686,12 +1686,12 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1728,12 +1728,12 @@
       </c>
       <c r="I32" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J32" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1770,12 +1770,12 @@
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1812,12 +1812,12 @@
       </c>
       <c r="I34" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J34" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1854,12 +1854,12 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1896,12 +1896,12 @@
       </c>
       <c r="I36" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J36" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1938,12 +1938,12 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -1980,12 +1980,12 @@
       </c>
       <c r="I38" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J38" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2022,12 +2022,12 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2064,12 +2064,12 @@
       </c>
       <c r="I40" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J40" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2106,12 +2106,12 @@
       </c>
       <c r="I41" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2148,12 +2148,12 @@
       </c>
       <c r="I42" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J42" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2190,12 +2190,12 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2232,12 +2232,12 @@
       </c>
       <c r="I44" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J44" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2274,12 +2274,12 @@
       </c>
       <c r="I45" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2316,12 +2316,12 @@
       </c>
       <c r="I46" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J46" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2358,12 +2358,12 @@
       </c>
       <c r="I47" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2400,12 +2400,12 @@
       </c>
       <c r="I48" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J48" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2442,12 +2442,12 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2484,12 +2484,12 @@
       </c>
       <c r="I50" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J50" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2526,12 +2526,12 @@
       </c>
       <c r="I51" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2568,12 +2568,12 @@
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J52" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2610,12 +2610,12 @@
       </c>
       <c r="I53" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2652,12 +2652,12 @@
       </c>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J54" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2694,12 +2694,12 @@
       </c>
       <c r="I55" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2736,12 +2736,12 @@
       </c>
       <c r="I56" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J56" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2778,12 +2778,12 @@
       </c>
       <c r="I57" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2820,12 +2820,12 @@
       </c>
       <c r="I58" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J58" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2862,12 +2862,12 @@
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2904,12 +2904,12 @@
       </c>
       <c r="I60" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2946,12 +2946,12 @@
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -2988,12 +2988,12 @@
       </c>
       <c r="I62" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J62" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="I63" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3072,12 +3072,12 @@
       </c>
       <c r="I64" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J64" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3114,12 +3114,12 @@
       </c>
       <c r="I65" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3156,12 +3156,12 @@
       </c>
       <c r="I66" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J66" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3198,12 +3198,12 @@
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3240,12 +3240,12 @@
       </c>
       <c r="I68" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J68" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3282,12 +3282,12 @@
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3324,12 +3324,12 @@
       </c>
       <c r="I70" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J70" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3366,12 +3366,12 @@
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3408,12 +3408,12 @@
       </c>
       <c r="I72" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J72" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3450,12 +3450,12 @@
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3492,12 +3492,12 @@
       </c>
       <c r="I74" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J74" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3534,12 +3534,12 @@
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3576,12 +3576,12 @@
       </c>
       <c r="I76" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J76" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3618,12 +3618,12 @@
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J77" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3660,12 +3660,12 @@
       </c>
       <c r="I78" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J78" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3702,12 +3702,12 @@
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3744,12 +3744,12 @@
       </c>
       <c r="I80" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J80" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3786,12 +3786,12 @@
       </c>
       <c r="I81" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J81" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3828,12 +3828,12 @@
       </c>
       <c r="I82" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J82" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3870,12 +3870,12 @@
       </c>
       <c r="I83" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J83" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3912,12 +3912,12 @@
       </c>
       <c r="I84" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J84" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3954,12 +3954,12 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J85" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -3996,12 +3996,12 @@
       </c>
       <c r="I86" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J86" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4038,12 +4038,12 @@
       </c>
       <c r="I87" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J87" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4080,12 +4080,12 @@
       </c>
       <c r="I88" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J88" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4122,12 +4122,12 @@
       </c>
       <c r="I89" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J89" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4164,12 +4164,12 @@
       </c>
       <c r="I90" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J90" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4206,12 +4206,12 @@
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J91" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4248,12 +4248,12 @@
       </c>
       <c r="I92" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J92" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4290,12 +4290,12 @@
       </c>
       <c r="I93" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J93" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4332,12 +4332,12 @@
       </c>
       <c r="I94" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J94" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4374,12 +4374,12 @@
       </c>
       <c r="I95" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J95" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4416,12 +4416,12 @@
       </c>
       <c r="I96" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J96" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4458,12 +4458,12 @@
       </c>
       <c r="I97" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J97" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4500,12 +4500,12 @@
       </c>
       <c r="I98" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J98" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4542,12 +4542,12 @@
       </c>
       <c r="I99" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J99" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4584,12 +4584,12 @@
       </c>
       <c r="I100" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J100" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4626,12 +4626,12 @@
       </c>
       <c r="I101" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J101" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4668,12 +4668,12 @@
       </c>
       <c r="I102" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J102" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4710,12 +4710,12 @@
       </c>
       <c r="I103" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J103" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4752,12 +4752,12 @@
       </c>
       <c r="I104" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J104" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4794,12 +4794,12 @@
       </c>
       <c r="I105" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J105" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4836,12 +4836,54 @@
       </c>
       <c r="I106" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="J106" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C107" s="6" t="n">
+        <v>2.898233</v>
+      </c>
+      <c r="D107" s="6" t="n">
+        <v>59.204081</v>
+      </c>
+      <c r="E107" s="6" t="n">
+        <v>56.19622</v>
+      </c>
+      <c r="F107" s="6" t="n">
+        <v>6.653023</v>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>Definitivo</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>INEGI — Encuesta Nacional de Ocupación y Empleo (ENOE/ENOEN)</t>
+        </is>
+      </c>
+      <c r="I107" s="7" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="J107" s="7" t="inlineStr">
+        <is>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4860,7 +4902,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H106"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4883,7 +4925,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fuente: INEGI — Encuesta Nacional de Ocupación y Empleo (ENOE/ENOEN) · Frecuencia: Trimestral · Unidad: millones de personas · Boletín: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf · Fecha de publicación: 24 de julio de 2026</t>
+          <t>Fuente: INEGI — Encuesta Nacional de Ocupación y Empleo (ENOE/ENOEN) · Frecuencia: Trimestral · Unidad: millones de personas · Boletín: https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf · Fecha de publicación: 27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4956,12 +4998,12 @@
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -4988,12 +5030,12 @@
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5020,12 +5062,12 @@
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5056,12 +5098,12 @@
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5088,12 +5130,12 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5120,12 +5162,12 @@
       </c>
       <c r="G10" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5156,12 +5198,12 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5188,12 +5230,12 @@
       </c>
       <c r="G12" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5220,12 +5262,12 @@
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5256,12 +5298,12 @@
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H14" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5330,12 @@
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5320,12 +5362,12 @@
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5356,12 +5398,12 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5388,12 +5430,12 @@
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5420,12 +5462,12 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5456,12 +5498,12 @@
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H20" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5488,12 +5530,12 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5520,12 +5562,12 @@
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H22" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5556,12 +5598,12 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5588,12 +5630,12 @@
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H24" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5620,12 +5662,12 @@
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5656,12 +5698,12 @@
       </c>
       <c r="G26" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H26" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5688,12 +5730,12 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5762,12 @@
       </c>
       <c r="G28" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H28" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5756,12 +5798,12 @@
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5788,12 +5830,12 @@
       </c>
       <c r="G30" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H30" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5820,12 +5862,12 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5856,12 +5898,12 @@
       </c>
       <c r="G32" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H32" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5888,12 +5930,12 @@
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5920,12 +5962,12 @@
       </c>
       <c r="G34" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H34" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5956,12 +5998,12 @@
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -5988,12 +6030,12 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H36" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6020,12 +6062,12 @@
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6056,12 +6098,12 @@
       </c>
       <c r="G38" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H38" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6088,12 +6130,12 @@
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6120,12 +6162,12 @@
       </c>
       <c r="G40" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H40" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6156,12 +6198,12 @@
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6188,12 +6230,12 @@
       </c>
       <c r="G42" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H42" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6220,12 +6262,12 @@
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6256,12 +6298,12 @@
       </c>
       <c r="G44" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H44" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6288,12 +6330,12 @@
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6320,12 +6362,12 @@
       </c>
       <c r="G46" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H46" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6356,12 +6398,12 @@
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6388,12 +6430,12 @@
       </c>
       <c r="G48" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H48" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6420,12 +6462,12 @@
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6456,12 +6498,12 @@
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H50" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6488,12 +6530,12 @@
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6520,12 +6562,12 @@
       </c>
       <c r="G52" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H52" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6556,12 +6598,12 @@
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6588,12 +6630,12 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H54" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6620,12 +6662,12 @@
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6656,12 +6698,12 @@
       </c>
       <c r="G56" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H56" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6688,12 +6730,12 @@
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6720,12 +6762,12 @@
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6756,12 +6798,12 @@
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6788,12 +6830,12 @@
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H60" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6820,12 +6862,12 @@
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6856,12 +6898,12 @@
       </c>
       <c r="G62" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H62" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6888,12 +6930,12 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6920,12 +6962,12 @@
       </c>
       <c r="G64" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H64" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6956,12 +6998,12 @@
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -6988,12 +7030,12 @@
       </c>
       <c r="G66" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H66" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7020,12 +7062,12 @@
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7056,12 +7098,12 @@
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H68" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7088,12 +7130,12 @@
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7120,12 +7162,12 @@
       </c>
       <c r="G70" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H70" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7156,12 +7198,12 @@
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7188,12 +7230,12 @@
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7220,12 +7262,12 @@
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7256,12 +7298,12 @@
       </c>
       <c r="G74" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H74" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7288,12 +7330,12 @@
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7320,12 +7362,12 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H76" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7356,12 +7398,12 @@
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7388,12 +7430,12 @@
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H78" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7420,12 +7462,12 @@
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7456,12 +7498,12 @@
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H80" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7488,12 +7530,12 @@
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7520,12 +7562,12 @@
       </c>
       <c r="G82" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H82" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7556,12 +7598,12 @@
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7588,12 +7630,12 @@
       </c>
       <c r="G84" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H84" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7620,12 +7662,12 @@
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7656,12 +7698,12 @@
       </c>
       <c r="G86" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H86" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7688,12 +7730,12 @@
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7720,12 +7762,12 @@
       </c>
       <c r="G88" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H88" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7756,12 +7798,12 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7788,12 +7830,12 @@
       </c>
       <c r="G90" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H90" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7820,12 +7862,12 @@
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7856,12 +7898,12 @@
       </c>
       <c r="G92" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H92" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7888,12 +7930,12 @@
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7920,12 +7962,12 @@
       </c>
       <c r="G94" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H94" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7956,12 +7998,12 @@
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -7988,12 +8030,12 @@
       </c>
       <c r="G96" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H96" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8020,12 +8062,12 @@
       </c>
       <c r="G97" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8056,12 +8098,12 @@
       </c>
       <c r="G98" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H98" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8088,12 +8130,12 @@
       </c>
       <c r="G99" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8120,12 +8162,12 @@
       </c>
       <c r="G100" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H100" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8156,12 +8198,12 @@
       </c>
       <c r="G101" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8188,12 +8230,12 @@
       </c>
       <c r="G102" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H102" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8220,12 +8262,12 @@
       </c>
       <c r="G103" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H103" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8256,12 +8298,12 @@
       </c>
       <c r="G104" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H104" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8288,12 +8330,12 @@
       </c>
       <c r="G105" s="7" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H105" s="7" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>
@@ -8320,12 +8362,44 @@
       </c>
       <c r="G106" s="9" t="inlineStr">
         <is>
-          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_07.pdf</t>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
         </is>
       </c>
       <c r="H106" s="9" t="inlineStr">
         <is>
-          <t>24 de julio de 2026</t>
+          <t>27 de agosto de 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>Jul 26</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="n">
+        <v>46204</v>
+      </c>
+      <c r="C107" s="10" t="n"/>
+      <c r="D107" s="11" t="n"/>
+      <c r="E107" s="7" t="inlineStr">
+        <is>
+          <t>Definitivo</t>
+        </is>
+      </c>
+      <c r="F107" s="7" t="inlineStr">
+        <is>
+          <t>INEGI — Encuesta Nacional de Ocupación y Empleo (ENOE/ENOEN)</t>
+        </is>
+      </c>
+      <c r="G107" s="7" t="inlineStr">
+        <is>
+          <t>https://www.inegi.org.mx/contenidos/saladeprensa/boletines/2026/iooe/IOE2026_08.pdf</t>
+        </is>
+      </c>
+      <c r="H107" s="7" t="inlineStr">
+        <is>
+          <t>27 de agosto de 2026</t>
         </is>
       </c>
     </row>

</xml_diff>